<commit_message>
Added in standards error column
</commit_message>
<xml_diff>
--- a/PIMMS v1.2/import folder/MPFAC HIF ES SIL peaks.xlsx
+++ b/PIMMS v1.2/import folder/MPFAC HIF ES SIL peaks.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Twins Project (2.24-)\Non-target work\Import Folder\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\PFAS-IMplementor-for-Mass-Spectrometry--PIMMS-\PIMMS v1.2\import folder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F9042E2-A5C4-4A5B-AC82-39A0CD5C911A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E47DD74-B1D3-46D3-BAC3-29ACE4381AA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{652C3A68-403A-4B28-96E6-555C4519F303}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{652C3A68-403A-4B28-96E6-555C4519F303}"/>
   </bookViews>
   <sheets>
     <sheet name="MPFAC-HIF-ES Peaks" sheetId="1" r:id="rId1"/>

</xml_diff>